<commit_message>
scan: seg0 2026-10-26 15:56 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq1_2026-10-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>67.22819401833083</v>
+        <v>67.22819398842594</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>50.98827078081172</v>
+        <v>50.98827085050917</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.885756429607231</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.1247669717314016</v>
+        <v>0.1247669717054427</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>74.65694148261387</v>
+        <v>74.65694168122968</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>35.20061183568823</v>
+        <v>35.20061196990339</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.509864838249063</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.178410070576341</v>
+        <v>0.1784100703946423</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>67.50565610259397</v>
+        <v>67.5056561594111</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>40.84737949354994</v>
+        <v>40.84737971132715</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.697540842941109</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.03878559625934105</v>
+        <v>0.03878559623338287</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>66.83291417447336</v>
+        <v>66.83291422716002</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>26.83188236739417</v>
+        <v>26.83188239631996</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>0.8012040686294437</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>75.90264241624436</v>
+        <v>75.90264246993375</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>67.32218148872418</v>
+        <v>67.32218159404157</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.675067735922812</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.7106369435236903</v>
+        <v>0.7106369429785833</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>881.1465846849743</v>
+        <v>881.1465846849742</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>25.9</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>61.21968079438652</v>
+        <v>61.21968084120295</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>31.86824647567126</v>
+        <v>31.86824649174469</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>4.318140680598007</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-0.01683316871074081</v>
+        <v>-0.0168331688535106</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>64.64530955491284</v>
+        <v>64.64530960569995</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>22.88550414344115</v>
+        <v>22.88550418193258</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>5.107305877482982</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.2264940050308146</v>
+        <v>0.2264940049918794</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>72.81261402898284</v>
+        <v>72.81261398142284</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>16.81551510010856</v>
+        <v>16.81551512012239</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>5.434070040980663</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.5360087806822283</v>
+        <v>0.5360087807028222</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>67.02608781183133</v>
+        <v>67.02608797022444</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>50.93368224852669</v>
+        <v>50.93368260422874</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.134148269745486</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-0.0452511197424359</v>
+        <v>-0.04525112026158373</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>75.48451859660825</v>
+        <v>75.48451856138273</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>44.7818591829032</v>
+        <v>44.78185920319464</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.7015148824678775</v>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>58.68973236823521</v>
+        <v>58.68973244246511</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>22.52493958528356</v>
+        <v>22.52493966124407</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.899879554683425</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.03134056231947421</v>
+        <v>-0.03134056241032546</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>63.94408705260311</v>
+        <v>63.94408716312676</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>33.41179717905271</v>
+        <v>33.41179720512135</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.6783956063873652</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1.147858199281586</v>
+        <v>1.147858198892192</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>66.41068528399984</v>
+        <v>66.41068530488567</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>37.8620539103713</v>
+        <v>37.86205394942604</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.4762559980374482</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>4.134197855375534</v>
+        <v>4.134197855115971</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>50.31850582068898</v>
+        <v>50.31850578639637</v>
       </c>
       <c r="I15" s="2" t="n">
         <v>34.34935146180015</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-0.4444131549050043</v>
+        <v>-0.4444131548530863</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>56.1484781941305</v>
+        <v>56.14847813983678</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>20.49943886509741</v>
+        <v>20.49943875578506</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.6430549803829058</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.03910150812958971</v>
+        <v>0.0391015081815056</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>48.88576558020389</v>
+        <v>48.88576560429723</v>
       </c>
       <c r="I17" s="2" t="n">
         <v>23.53005489333985</v>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>625.3482834581496</v>
+        <v>625.3482834581494</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>14.55</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>54.92073618613777</v>
+        <v>54.92073615385726</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>16.6983919890933</v>
+        <v>16.69839206628611</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.5315720086149386</v>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>620.29575185482</v>
+        <v>620.2957518548201</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>13.9</v>
@@ -1456,7 +1456,7 @@
         <v>52.57465550717582</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>21.89920479298087</v>
+        <v>21.89920482240279</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.3663848025068586</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-0.01318895398077691</v>
+        <v>-0.01318895399375591</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>56.56586679743685</v>
+        <v>56.56586678628602</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>43.51910231715581</v>
+        <v>43.51910239281162</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.052114640484283</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-1.577043196913085</v>
+        <v>-1.577043197094817</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>54.51453730355608</v>
+        <v>54.51453742783769</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>19.9678902238398</v>
+        <v>19.96789041810956</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.9038954883700848</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.02756989543045099</v>
+        <v>0.02756989530065895</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>44.19179884816317</v>
+        <v>44.19179891154599</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>31.8314960356828</v>
+        <v>31.83149605483471</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>1.186265452776034</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.01087099059645795</v>
+        <v>0.01087099060943742</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>47.16151897971363</v>
+        <v>47.16151896894623</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>41.36980284747396</v>
+        <v>41.36980294127662</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.4620147805487044</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.1796110411469446</v>
+        <v>-0.1796110411495419</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1721,7 +1721,7 @@
         <v>64.61188617286926</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>29.49881619415126</v>
+        <v>29.49881620630818</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.8017099990846154</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>52.15532288858483</v>
+        <v>52.15532367404824</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>12.11643028644397</v>
+        <v>12.1164318243229</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.2489099817051164</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.07544777278270004</v>
+        <v>0.07544776766909794</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>47.28923752711714</v>
+        <v>47.28923757597592</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>39.49940665830184</v>
+        <v>39.49940682742422</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.5643919099444266</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>-0.9097498069136005</v>
+        <v>-0.909749807158271</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>545.7225723372153</v>
+        <v>545.7225723372154</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>73.8</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>51.61101266922207</v>
+        <v>51.61101265319471</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>38.3520491998043</v>
+        <v>38.35204925791102</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.6013248262975751</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.5021899417599913</v>
+        <v>-0.5021899417989282</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>535.7105702311541</v>
+        <v>535.7105702311542</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>43.15</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>48.43272904964675</v>
+        <v>48.43272907025969</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>10.0096741267398</v>
+        <v>10.0096741684959</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.9006456250374378</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.01340311611296929</v>
+        <v>0.01340311608700734</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>51.80010973807624</v>
+        <v>51.80010964121629</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>45.89465837480962</v>
+        <v>45.89465848349738</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.5490835262969375</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-0.04145491806589163</v>
+        <v>-0.04145491802955109</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>55.1794265490582</v>
+        <v>55.1794262083976</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>26.34376177058579</v>
+        <v>26.34376179738685</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.4785622234440209</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.1284552826026084</v>
+        <v>0.1284552829919584</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>54.47681658305314</v>
+        <v>54.47681661908713</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>37.83509269077872</v>
+        <v>37.83509276485403</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.5334352961232455</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.01415644551058193</v>
+        <v>0.01415644547164779</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2145,7 +2145,7 @@
         <v>55.11004129299651</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>23.35014564415632</v>
+        <v>23.35014579607236</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.8490513455903952</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.2353773387000584</v>
+        <v>-0.2353773390115483</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>517.5159755642122</v>
+        <v>517.5159755642121</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>846</v>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>42.08095388467736</v>
+        <v>42.08095386568425</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>31.95696279954685</v>
+        <v>31.9569628647352</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.8192230758207769</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-25.0275619679547</v>
+        <v>-25.02756196951225</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>43.43331045476441</v>
+        <v>43.43331054955119</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>23.18524993762747</v>
+        <v>23.1852499836581</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.5782598888956022</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>41.03846279133447</v>
+        <v>41.03846305375814</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>13.76842119257366</v>
+        <v>13.76842122587007</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>3.710012438565919</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-0.02153990639402967</v>
+        <v>-0.02153990643296569</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>38.6869199916101</v>
+        <v>38.68692009798401</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>11.42811229698812</v>
+        <v>11.4281123547563</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.6214000071743462</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.8305585320714264</v>
+        <v>-0.8305585337586323</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>480.930952705536</v>
+        <v>480.9309527055358</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>21.75</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>43.03933676744486</v>
+        <v>43.03933682502424</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>21.01873653586321</v>
+        <v>21.0187365789877</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.7439184876399714</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.0154379133416423</v>
+        <v>0.01543791328972619</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>43.31295781375929</v>
+        <v>43.31295776200458</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>37.7831434588695</v>
+        <v>37.78314352969066</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.5280489279729099</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.0825021932778363</v>
+        <v>-0.08250219329081446</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>47.63970805635945</v>
+        <v>47.63970803071238</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>24.46382271990138</v>
+        <v>24.46382276920145</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.4005305714480796</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.0994551885893783</v>
+        <v>-0.09945518862831493</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>461.2596177740492</v>
+        <v>461.2596177740485</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>20</v>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>50.53173033559301</v>
+        <v>50.53173034343114</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>10.6238493478604</v>
+        <v>10.62384955175526</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>2.851818566293085</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.07044048162124739</v>
+        <v>0.07044048147848354</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>45.90484693019192</v>
+        <v>45.90484707074836</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>16.09166015874677</v>
+        <v>16.09166021232069</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.9830428177862458</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.02387868821441951</v>
+        <v>0.02387868795486116</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>47.91113729098156</v>
+        <v>47.91113739662757</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>20.7706201131799</v>
+        <v>20.77062009857078</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1.046944844780225</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.2491873195380336</v>
+        <v>0.2491873192784642</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>45.52996769037252</v>
+        <v>45.52996767493394</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>28.72846170757203</v>
+        <v>28.72846159659593</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.5969970290769615</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.07895135550931476</v>
+        <v>-0.07895135549633486</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>53.48868763967705</v>
+        <v>53.48868767907326</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>17.83851628019204</v>
+        <v>17.83851637131479</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.94351239308079</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.01672001997694503</v>
+        <v>0.01672001995098953</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>48.90119524052107</v>
+        <v>48.90119524669444</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>15.21305720695588</v>
+        <v>15.21305716388626</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.9174516046541222</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.07487907053995242</v>
+        <v>-0.07487907074761091</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>40.5662988135626</v>
+        <v>40.56629876217429</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>31.68460792312481</v>
+        <v>31.6846080064185</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.7366654226485709</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.1081335552827524</v>
+        <v>-0.1081335552697738</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>58.47485539775608</v>
+        <v>58.47485537756555</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>64.22641136979226</v>
+        <v>64.22641151136584</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.1763728741855054</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>51.61039192268831</v>
+        <v>51.61039199843174</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>13.1423371512287</v>
+        <v>13.14233716754401</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.5422154285748083</v>
@@ -3046,7 +3046,7 @@
         <v>48.07826756401787</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>13.37057198700673</v>
+        <v>13.37057198700672</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.3545110359982702</v>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>426.2256036612502</v>
+        <v>426.2256036612503</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>26.5</v>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>48.37519985326762</v>
+        <v>48.37519996138513</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>13.52240630057613</v>
+        <v>13.52240632268671</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>1.036533289575128</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.08582274837837976</v>
+        <v>0.08582274819667798</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>46.66568627613604</v>
+        <v>46.66568635272273</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>29.72973539784932</v>
+        <v>29.72973555512544</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.2241673381767101</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.1746697746732524</v>
+        <v>-0.1746697747641023</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>43.7304750753824</v>
+        <v>43.73047503588652</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>34.41011017552491</v>
+        <v>34.410110244324</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.5287290176459353</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.09724607069696029</v>
+        <v>-0.09724607070993924</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>52.62412261036246</v>
+        <v>52.6241226032864</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>6.444766285013309</v>
+        <v>6.444766288243534</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.4875341668806329</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.2529556236433477</v>
+        <v>-0.2529556235914483</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>47.43459299079519</v>
+        <v>47.4345929121767</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>36.48648910387239</v>
+        <v>36.48648929627024</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.4503480288655173</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.05008545236776255</v>
+        <v>-0.05008545235478354</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>53.39231253641537</v>
+        <v>53.39231258147935</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>17.52592621661223</v>
+        <v>17.52592628712955</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>1.110544920475465</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.01060223128731803</v>
+        <v>0.01060223122242689</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>399.3025367340296</v>
+        <v>399.3025367340298</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>10.3</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>43.39820073397857</v>
+        <v>43.39820066028695</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>23.09991949363018</v>
+        <v>23.09991959203426</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1.690104392507155</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.02316421767544768</v>
+        <v>0.02316421768842664</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>39.32029416923925</v>
+        <v>39.32029422982587</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>44.38443207812463</v>
+        <v>44.38443212941924</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.26527737954334</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.03832927483297471</v>
+        <v>0.03832927484595461</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.47628258805543</v>
+        <v>51.47628324819883</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>9.195139657620912</v>
+        <v>9.195140867425428</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.213837046724031</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.06219018997165694</v>
+        <v>-0.06219019325526491</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>388.7671418522369</v>
+        <v>388.7671418522368</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>18.85</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>34.97952203631272</v>
+        <v>34.97952221959444</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>44.88680352163931</v>
+        <v>44.88680352530255</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1.444803384559349</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.0007838578730914036</v>
+        <v>-0.0007838579898996334</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>384.4145656427831</v>
+        <v>384.4145656427888</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>98.59999999999999</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>40.93268048618865</v>
+        <v>40.93268069948992</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>11.74183229638204</v>
+        <v>11.74183240172536</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.7215689761067196</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.4176754123772879</v>
+        <v>-0.417675413804938</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>51.10893499769771</v>
+        <v>51.10893496109806</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>19.23056757529915</v>
+        <v>19.23056751969887</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>1.107740551194117</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.008362932128092672</v>
+        <v>0.008362932024265073</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>379.0206616479385</v>
+        <v>379.0206616479383</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>31</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>49.60348735734944</v>
+        <v>49.60348738275516</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>11.84462246610018</v>
+        <v>11.84462254659206</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>1.268534588509361</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.03824517284626756</v>
+        <v>-0.0382451729630765</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>375.7268237757937</v>
+        <v>375.7268237757938</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>17</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>43.05829126220716</v>
+        <v>43.05829138163871</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>12.8267462131565</v>
+        <v>12.82674628956885</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.4001182870078424</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.003922198414267282</v>
+        <v>0.003922198388312065</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>42.37011668304041</v>
+        <v>42.3701167487967</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>8.319428195744438</v>
+        <v>8.319427966574546</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.4600557741757824</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.2191739783363484</v>
+        <v>0.2191739813214595</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>50.73405679072533</v>
+        <v>50.73405691926826</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>7.973975386292214</v>
+        <v>7.973975423213428</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.5975139833209947</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.0004004809074422515</v>
+        <v>0.0004004808814840428</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>44.89434108506562</v>
+        <v>44.89434105419756</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>34.77860012191497</v>
+        <v>34.7786001449895</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.5454585161494226</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.0738363473651118</v>
+        <v>-0.07383634735732553</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>346.6733874472961</v>
+        <v>346.6733874472962</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>26.65</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>49.59765327557657</v>
+        <v>49.5976532914535</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>28.4395936734038</v>
+        <v>28.43959363612493</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.5393660494386591</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.05352941674292044</v>
+        <v>0.05352941662611273</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>44.43472543376139</v>
+        <v>44.43472540499618</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>16.63724608769352</v>
+        <v>16.63724609672827</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>3.841408098733572</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.004043074459428808</v>
+        <v>-0.004043074446452521</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>54.76490306619252</v>
+        <v>54.76490287283215</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>8.820709995351043</v>
+        <v>8.820709964488103</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.3444450285100885</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>30.27544526690903</v>
+        <v>30.2754452998782</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>28.26196199971221</v>
+        <v>28.26196207568031</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.7234782411867646</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.005899539086103342</v>
+        <v>0.005899539078315641</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>43.36351037534183</v>
+        <v>43.36351028964666</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>16.19488793105122</v>
+        <v>16.19488793326233</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.808491582247074</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.02617305415082732</v>
+        <v>-0.02617305409891257</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>41.1051390941152</v>
+        <v>41.10513916883784</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>27.25126430947455</v>
+        <v>27.25126446151379</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.9228546604900439</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.01251598976722607</v>
+        <v>-0.01251598993595038</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>41.64187541071813</v>
+        <v>41.64187539323201</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>15.9029000964332</v>
+        <v>15.90290027438911</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.4808313018780662</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.01251024861584429</v>
+        <v>-0.01251024861324925</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>37.30382887658166</v>
+        <v>37.30382884942652</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>14.48436564886853</v>
+        <v>14.48436563941315</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1.663891804908274</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.06593604110046239</v>
+        <v>-0.06593604117833188</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>47.80496242511996</v>
+        <v>47.80496237772534</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>32.49655271958042</v>
+        <v>32.49655268292496</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.407632821778858</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.04664076744104809</v>
+        <v>-0.04664076745402679</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>33.01850191987452</v>
+        <v>33.01850203109586</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>30.00260833514157</v>
+        <v>30.00260844242966</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1.097233452453498</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.06424678548464469</v>
+        <v>-0.06424678573124165</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>45.35651936976606</v>
+        <v>45.35651942139969</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>33.07498640195481</v>
+        <v>33.07498638671085</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.3913103384926285</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.04513001617764176</v>
+        <v>-0.04513001619581303</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>38.48702343291328</v>
+        <v>38.48702325705609</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>7.617536348053889</v>
+        <v>7.617536382793276</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.6271837785975587</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.009527175774447116</v>
+        <v>0.00952717578742529</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>34.86981328212447</v>
+        <v>34.86981319594247</v>
       </c>
       <c r="I79" s="2" t="n">
         <v>25.36638529354557</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>34.23089086729462</v>
+        <v>34.23088979970008</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>18.41097726197723</v>
+        <v>18.41097811400233</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.7588313416947114</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.006374188734929884</v>
+        <v>0.00637418885173828</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>47.12656667669876</v>
+        <v>47.12656670682107</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>14.17372294326239</v>
+        <v>14.17372298714401</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.9979275133066693</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.003183945421184692</v>
+        <v>0.003183945382247713</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>38.48273909190718</v>
+        <v>38.48273887761444</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>7.946364096848186</v>
+        <v>7.9463645255898</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>1.141736795086661</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.02105877539483614</v>
+        <v>0.02105877570632486</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>50.37570354983596</v>
+        <v>50.37570355650195</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>8.071739521147883</v>
+        <v>8.071739603631645</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>1.591717518967429</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.273757593606871</v>
+        <v>0.2737575935030396</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>34.63655180391633</v>
+        <v>34.63655212079985</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>13.61785347832587</v>
+        <v>13.61785360486242</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.992951684169262</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.07171242524689847</v>
+        <v>-0.07171242537668543</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>35.74218418674596</v>
+        <v>35.74218414138525</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>11.12301220062339</v>
+        <v>11.12301228248422</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>1.760919502465495</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.01614659393983846</v>
+        <v>-0.01614659393724376</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>280.8215544552968</v>
+        <v>280.8215544552973</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>14.9</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>36.44424957313118</v>
+        <v>36.44424994528642</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>17.67498874108724</v>
+        <v>17.67498879254004</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.5843450739975848</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.007545946936837265</v>
+        <v>-0.007545946962794772</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>48.55393283862234</v>
+        <v>48.55393282858574</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>19.11615589845732</v>
+        <v>19.11615594113584</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.2529138567877762</v>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>278.5477045692471</v>
+        <v>278.5477045692472</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>13.05</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>36.26359413417264</v>
+        <v>36.26359385099953</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>36.43133900512838</v>
+        <v>36.43134016052537</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.110804882276412</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.007032436208796455</v>
+        <v>-0.007032436169860101</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>275.80856825208</v>
+        <v>275.8085682520794</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>9.859999999999999</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>40.88061474972265</v>
+        <v>40.88061330824178</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>19.32283006700711</v>
+        <v>19.32283039697867</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.9656777798966892</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.002733308688644874</v>
+        <v>-0.002733308623751617</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>272.1628941739328</v>
+        <v>272.1628941739327</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>17.35</v>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>43.43434984029913</v>
+        <v>43.43435007362613</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>16.82255517268307</v>
+        <v>16.82255521365153</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>1.169022783709383</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.04150184483052016</v>
+        <v>0.04150184485276265</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>30.25948870534828</v>
+        <v>30.2594886590818</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>34.58904658987375</v>
+        <v>34.58904658087221</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.6038300506478742</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>48.73350234500433</v>
+        <v>48.73350263634344</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>12.06062427980989</v>
+        <v>12.06062426556887</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.2324904627064758</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.0004678325356735243</v>
+        <v>0.0004678324837585519</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>269.6913430748821</v>
+        <v>269.691343074882</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>15.3</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>35.73061798298103</v>
+        <v>35.73061809196055</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>30.35315962862844</v>
+        <v>30.35315976877381</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>1.253583202524372</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.02073921303832876</v>
+        <v>-0.02073921310322206</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,7 +5428,7 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>40.22978147575908</v>
+        <v>40.2297815087816</v>
       </c>
       <c r="I94" s="2" t="n">
         <v>40.17210484007352</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.02320298581588753</v>
+        <v>0.0232029858029085</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>255.6636975973335</v>
+        <v>255.6636975973329</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>63.5</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>37.04555230374353</v>
+        <v>37.04555218429955</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>15.17341360682296</v>
+        <v>15.17341359534782</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.3550157074723045</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.2656956510363521</v>
+        <v>-0.2656956509584859</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5537,7 +5537,7 @@
         <v>50.99084933536099</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>13.7977472693179</v>
+        <v>13.79774724240975</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>1.009326928468627</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.3789605355343183</v>
+        <v>0.3789605355213391</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>247.0535719787309</v>
+        <v>247.0535719787305</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>69.90000000000001</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>44.13305884213477</v>
+        <v>44.13305890940874</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>13.70675871013541</v>
+        <v>13.70675867097003</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>1.947212138697003</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.01770878511476737</v>
+        <v>0.01770878467349235</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>31.78735351417725</v>
+        <v>31.78735427169219</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>24.10910253017152</v>
+        <v>24.10910258687021</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.8609879271902744</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.0827839458783165</v>
+        <v>-0.08278394642341602</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>46.32820835490458</v>
+        <v>46.32820850865157</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>13.4304674303655</v>
+        <v>13.43046753543922</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4522391118085424</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.00430651056415611</v>
+        <v>-0.004306510590113166</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>38.27339323710818</v>
+        <v>38.27339308707172</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>18.31161572055116</v>
+        <v>18.31161572625699</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.6835417548362436</v>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>234.3729286086376</v>
+        <v>234.3729286086362</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>32.05</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>37.1768262506079</v>
+        <v>37.17682643631351</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>10.08564669800517</v>
+        <v>10.08564701099007</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.7015852638147142</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.03795846211734499</v>
+        <v>-0.03795846226011274</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>232.7062305274775</v>
+        <v>232.7062305274769</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>96.7</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>31.06818699288814</v>
+        <v>31.06818707941413</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>18.6804090335585</v>
+        <v>18.68040907923018</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>1.711676728001756</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.3157175432616578</v>
+        <v>-0.3157175437548441</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>231.6225511311858</v>
+        <v>231.6225511311849</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>615</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>33.3021436707953</v>
+        <v>33.30214368564765</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>12.71618485340681</v>
+        <v>12.71618488121825</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5237464880521181</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-7.221732680277878</v>
+        <v>-7.221732687026851</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>41.53060149759695</v>
+        <v>41.53060187775376</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>24.7414287256596</v>
+        <v>24.7414289684885</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.4976793908482958</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.05860629733813769</v>
+        <v>-0.05860629757175465</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6014,7 +6014,7 @@
         <v>51.30613010717237</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>8.699330794350457</v>
+        <v>8.699330880273015</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.534455435045157</v>
@@ -6064,7 +6064,7 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>38.00230958774962</v>
+        <v>38.00230946826648</v>
       </c>
       <c r="I106" s="2" t="n">
         <v>17.1794584639681</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.003937246013506521</v>
+        <v>0.003937246065421091</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>42.23756923185449</v>
+        <v>42.23756932353022</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>9.796564228807661</v>
+        <v>9.796564315084856</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.8919521866451359</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.6151077118624446</v>
+        <v>-0.6151077143283727</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>216.5131984072283</v>
+        <v>216.5131984072286</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>13.3</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>39.13823099058795</v>
+        <v>39.13823110943726</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>12.03879514806371</v>
+        <v>12.03879517598908</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>1.036579126426111</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.001762770061251223</v>
+        <v>0.001762770009335432</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>47.08398958909182</v>
+        <v>47.08398949244717</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>7.494613851272913</v>
+        <v>7.494613851280223</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.7250902417192936</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.009910535291324934</v>
+        <v>0.009910535161537462</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>201.2126428627774</v>
+        <v>201.2126428627769</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>26</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>35.17635308601176</v>
+        <v>35.17635284514378</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>31.24519957971321</v>
+        <v>31.24519962925976</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.3988081913507854</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.009387731286727874</v>
+        <v>0.00938773146843086</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>194.9523194066126</v>
+        <v>194.9523194066122</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>39.95</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>43.65617295722609</v>
+        <v>43.65617313912831</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.56211267146425</v>
+        <v>17.56211252246812</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.5312389084996308</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.01970664848514056</v>
+        <v>0.01970664813471337</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>193.7034867605874</v>
+        <v>193.7034867605876</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>28.9</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>38.25111979138109</v>
+        <v>38.251120029319</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>22.97816376004682</v>
+        <v>22.97816382511045</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.5314132171035814</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.3378993240909592</v>
+        <v>-0.3378993239871319</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>192.9307045529359</v>
+        <v>192.9307045529357</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>9.710000000000001</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.01691312566274495</v>
+        <v>-0.01691312567572451</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>38.32101732290195</v>
+        <v>38.3210174005151</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>21.88645094564079</v>
+        <v>21.88645097900668</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.001584990708859</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.01417395940755704</v>
+        <v>-0.01417395944130147</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6544,7 +6544,7 @@
         <v>40.21898436341603</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>19.15769520255517</v>
+        <v>19.15769523305918</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.1910303369452782</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.01499404686367239</v>
+        <v>0.01499404685069336</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.89574361894764</v>
+        <v>39.8957435396395</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>22.60886461612286</v>
+        <v>22.60886457362271</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.5399184266849736</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.09427439949499988</v>
+        <v>-0.0942743995079792</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>182.9010162276014</v>
+        <v>182.901016227601</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>6.22</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>37.36424643908072</v>
+        <v>37.36424647422256</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>23.51100450974235</v>
+        <v>23.51100455219949</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>1.122346288879889</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.01097314849241471</v>
+        <v>-0.01097314850539313</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>181.8618183480429</v>
+        <v>181.8618183480426</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>74.3</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>20.77512246992806</v>
+        <v>20.77512345552299</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>36.12172669326548</v>
+        <v>36.12172657205576</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.7811844471055056</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.306433995964742</v>
+        <v>-0.3064339964838934</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>172.6220656043152</v>
+        <v>172.622065604318</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>12</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>40.41731726077874</v>
+        <v>40.41731719505214</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>20.99784951340072</v>
+        <v>20.99784949065089</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.9062851370223991</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.05279314742536149</v>
+        <v>-0.05279314737344756</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>38.74514950152395</v>
+        <v>38.74514951413121</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>17.09814371727719</v>
+        <v>17.09814368084951</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.1507890554741108</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-1.040451370784145</v>
+        <v>-1.040451370874996</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>159.8815429873118</v>
+        <v>159.8815429873115</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>20.2</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>50.06999577437925</v>
+        <v>50.06999611718037</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>5.946343943890253</v>
+        <v>5.946345208951548</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.5098654521723434</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.2266480968154221</v>
+        <v>0.2266480925937485</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>158.3932473135707</v>
+        <v>158.39324731357</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>9.01</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>32.40390741238264</v>
+        <v>32.40390734905704</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>15.84219308720742</v>
+        <v>15.84219300251613</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>1.381537630934448</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.02329689748786888</v>
+        <v>-0.02329689750084775</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>43.58614453866051</v>
+        <v>43.58614458480404</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>15.99865271575751</v>
+        <v>15.99865273214649</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.7138346245074088</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.04832510580186766</v>
+        <v>0.04832510574995136</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>42.95216515094675</v>
+        <v>42.95216474024279</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>15.94059430660055</v>
+        <v>15.94059467302017</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.3061135049663243</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.02715903383953844</v>
+        <v>0.02715903398230293</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>139.4856444413946</v>
+        <v>139.4856444413938</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>18.65</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>38.71151270596647</v>
+        <v>38.71151293968626</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>10.45389297204655</v>
+        <v>10.4538930990547</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.6394762684124387</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.002725307163337021</v>
+        <v>-0.002725307383973807</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>42.24321412130227</v>
+        <v>42.24321417403042</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>13.37833833198464</v>
+        <v>13.37833829015054</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.4283024881512028</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>0.003163794731219943</v>
+        <v>0.003163794723434196</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7163,7 +7163,7 @@
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>139.3426903358456</v>
+        <v>139.3426903358455</v>
       </c>
       <c r="E127" s="2" t="n">
         <v>0</v>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>8.101614096073149</v>
+        <v>8.101614084452024</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>32.2621861209558</v>
+        <v>32.26218604406749</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.08126407941833376</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.632821361759434</v>
+        <v>-0.6328213617388382</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>44.76535376608174</v>
+        <v>44.76535378377109</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>6.053047155210829</v>
+        <v>6.053047195481095</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.8043434055369213</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>-0.02149349948105486</v>
+        <v>-0.02149349949403238</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>35.60669345096761</v>
+        <v>35.60669350462861</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>21.45247890136554</v>
+        <v>21.45247887624866</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>0.3759249138092666</v>
@@ -7301,7 +7301,7 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>-0.03526027506355722</v>
+        <v>-0.0352602752841959</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7322,7 +7322,7 @@
         <v/>
       </c>
       <c r="D130" s="2" t="n">
-        <v>105.1629217276463</v>
+        <v>105.1629217276462</v>
       </c>
       <c r="E130" s="2" t="n">
         <v>35.2</v>
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>36.68310695845339</v>
+        <v>36.68310713789047</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>13.32351286118778</v>
+        <v>13.32351274331679</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.8476287377514268</v>
@@ -7354,7 +7354,7 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>-0.01876654601962796</v>
+        <v>-0.01876654633111702</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>42.86656463493487</v>
+        <v>42.86656468197072</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>17.2902323064675</v>
+        <v>17.2902323758677</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.4184158987861103</v>
@@ -7407,7 +7407,7 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>0.0135298723067625</v>
+        <v>0.01352987222888691</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
@@ -7428,7 +7428,7 @@
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>84.39037585176544</v>
+        <v>84.39037585176541</v>
       </c>
       <c r="E132" s="2" t="n">
         <v>27.6</v>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>37.83218395728447</v>
+        <v>37.83218397245656</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>17.80643324171685</v>
+        <v>17.80643321058857</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.7334442338185182</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>-0.009365828989417624</v>
+        <v>-0.009365829002395354</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7481,7 +7481,7 @@
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>83.83811406728185</v>
+        <v>83.83811406728192</v>
       </c>
       <c r="E133" s="2" t="n">
         <v>0</v>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>37.10901102618477</v>
+        <v>37.10901102455061</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>8.465557671708474</v>
+        <v>8.465557602412245</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>0.01393954882326975</v>

</xml_diff>

<commit_message>
scan: seg0 2026-10-27 00:10 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq1_2026-10-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>67.22819398842594</v>
+        <v>67.22819406826662</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>50.98827085050917</v>
+        <v>50.98827114508993</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.885756429607231</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.1247669717054427</v>
+        <v>0.1247669716353623</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>74.65694168122968</v>
+        <v>74.65694170885359</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>35.20061196990339</v>
+        <v>35.20061201114412</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.509864838249063</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.1784100703946423</v>
+        <v>0.1784100703806283</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>67.5056561594111</v>
+        <v>67.50565622059881</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>40.84737971132715</v>
+        <v>40.84737976118824</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.697540842941109</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.03878559623338287</v>
+        <v>0.03878559621936713</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>66.83291422716002</v>
+        <v>66.83291412754593</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>26.83188239631996</v>
+        <v>26.83188237953689</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>0.8012040686294437</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.4582317267078517</v>
+        <v>0.4582317269321299</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>75.90264246993375</v>
+        <v>75.90264252951931</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>67.32218159404157</v>
+        <v>67.32218159008508</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.675067735922812</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.7106369429785833</v>
+        <v>0.7106369427543093</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>881.1465846849742</v>
+        <v>881.1465846849743</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>25.9</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>61.21968084120295</v>
+        <v>61.21968087208622</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>31.86824649174469</v>
+        <v>31.86824651282204</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>4.318140680598007</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-0.0168331688535106</v>
+        <v>-0.0168331688955593</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>64.64530960569995</v>
+        <v>64.64530961413328</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>22.88550418193258</v>
+        <v>22.88550425046362</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>5.107305877482982</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.2264940049918794</v>
+        <v>0.2264940050058953</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>72.81261398142284</v>
+        <v>72.81261403264131</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>16.81551512012239</v>
+        <v>16.81551520788351</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>5.434070040980663</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.5360087807028222</v>
+        <v>0.53600878061385</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>67.02608797022444</v>
+        <v>67.02608801513507</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>50.93368260422874</v>
+        <v>50.93368264617315</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.134148269745486</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-0.04525112026158373</v>
+        <v>-0.04525112034568712</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.09727343412723777</v>
+        <v>0.09727343411322048</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>58.68973244246511</v>
+        <v>58.68973247454434</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>22.52493966124407</v>
+        <v>22.52493964712873</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.899879554683425</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.03134056241032546</v>
+        <v>-0.03134056242434258</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>63.94408716312676</v>
+        <v>63.94408747784205</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>33.41179720512135</v>
+        <v>33.41179713616474</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.6783956063873652</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1.147858198892192</v>
+        <v>1.14785819931272</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>66.41068530488567</v>
+        <v>66.41068536176695</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>37.86205394942604</v>
+        <v>37.86205389217329</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.4762559980374482</v>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>50.31850578639637</v>
+        <v>50.31850580347449</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>34.34935146180015</v>
+        <v>34.3493513625862</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.5959525816474684</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-0.4444131548530863</v>
+        <v>-0.4444131551614587</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>56.14847813983678</v>
+        <v>56.14847807043574</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>20.49943875578506</v>
+        <v>20.49943876514065</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.6430549803829058</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.0391015081815056</v>
+        <v>0.03910150819552225</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>48.88576560429723</v>
+        <v>48.88576557835056</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>23.53005489333985</v>
+        <v>23.53005504621703</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.784399689079536</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-0.01664002015503629</v>
+        <v>-0.01664002014102071</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>625.3482834581494</v>
+        <v>625.3482834581496</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>14.55</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>54.92073615385726</v>
+        <v>54.92073624568924</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>16.69839206628611</v>
+        <v>16.69839202725624</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.5315720086149386</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.02338600392438938</v>
+        <v>0.02338600391037216</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>52.57465550717582</v>
+        <v>52.5746555263542</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>21.89920482240279</v>
+        <v>21.89920472552367</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.3663848025068586</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-0.01318895399375591</v>
+        <v>-0.01318895400777273</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>56.56586678628602</v>
+        <v>56.56586679892664</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>43.51910239281162</v>
+        <v>43.5191025502931</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.052114640484283</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-1.577043197094817</v>
+        <v>-1.577043197823663</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>54.51453742783769</v>
+        <v>54.51453744845245</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>19.96789041810956</v>
+        <v>19.96789044440318</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.9038954883700848</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.02756989530065895</v>
+        <v>0.02756989531468068</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>44.19179891154599</v>
+        <v>44.1917987821331</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>31.83149605483471</v>
+        <v>31.83149610268009</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>1.186265452776034</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.01087099060943742</v>
+        <v>0.01087099065148765</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>47.16151896894623</v>
+        <v>47.16151896430795</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>41.36980294127662</v>
+        <v>41.36980289120726</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.4620147805487044</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.1796110411495419</v>
+        <v>-0.1796110411803773</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>64.61188617286926</v>
+        <v>64.61188614565484</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>29.49881620630818</v>
+        <v>29.4988162359017</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.8017099990846154</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>52.15532367404824</v>
+        <v>52.15532327036512</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>12.1164318243229</v>
+        <v>12.11643055802605</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.2489099817051164</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.07544776766909794</v>
+        <v>0.07544777319178941</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>47.28923757597592</v>
+        <v>47.28923759720881</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>39.49940682742422</v>
+        <v>39.49940680673548</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.5643919099444266</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>-0.909749807158271</v>
+        <v>-0.9097498070381662</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>545.7225723372154</v>
+        <v>545.7225723372153</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>73.8</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>51.61101265319471</v>
+        <v>51.61101266613989</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>38.35204925791102</v>
+        <v>38.35204924639145</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.6013248262975751</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.5021899417989282</v>
+        <v>-0.5021899420091787</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>535.7105702311542</v>
+        <v>535.710570231155</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>43.15</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>48.43272907025969</v>
+        <v>48.43272913894283</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>10.0096741684959</v>
+        <v>10.00967414039615</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.9006456250374378</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.01340311608700734</v>
+        <v>0.01340311611504297</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>51.80010964121629</v>
+        <v>51.80010966964143</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>45.89465848349738</v>
+        <v>45.89465832465102</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.5490835262969375</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-0.04145491802955109</v>
+        <v>-0.04145491808561985</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>55.1794262083976</v>
+        <v>55.17942632238739</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>26.34376179738685</v>
+        <v>26.34376177125698</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.4785622234440209</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.1284552829919584</v>
+        <v>0.128455282431282</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>54.47681661908713</v>
+        <v>54.4768165802813</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>37.83509276485403</v>
+        <v>37.83509284711179</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.5334352961232455</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>55.11004129299651</v>
+        <v>55.1100413764452</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>23.35014579607236</v>
+        <v>23.35014599621263</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.8490513455903952</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.2353773390115483</v>
+        <v>-0.2353773393479477</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>42.08095386568425</v>
+        <v>42.08095392126996</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>31.9569628647352</v>
+        <v>31.95696305840941</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.8192230758207769</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-25.02756196951225</v>
+        <v>-25.02756197329683</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>43.43331054955119</v>
+        <v>43.43331039522106</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>23.1852499836581</v>
+        <v>23.18525008313585</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.5782598888956022</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.02834004245045718</v>
+        <v>0.02834004253455696</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>41.03846305375814</v>
+        <v>41.03846319352465</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>13.76842122587007</v>
+        <v>13.76842115646427</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>3.710012438565919</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-0.02153990643296569</v>
+        <v>-0.02153990634886209</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>495.7151263707709</v>
+        <v>495.7151263707708</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>160</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>38.68692009798401</v>
+        <v>38.68692035179406</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>11.4281123547563</v>
+        <v>11.42811246218118</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.6214000071743462</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.8305585337586323</v>
+        <v>-0.8305585345996461</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>43.03933682502424</v>
+        <v>43.03933687304897</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>21.0187365789877</v>
+        <v>21.01873652113024</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.7439184876399714</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.01543791328972619</v>
+        <v>0.01543791327570723</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>43.31295776200458</v>
+        <v>43.31295803084129</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>37.78314352969066</v>
+        <v>37.78314363574849</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.5280489279729099</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.08250219329081446</v>
+        <v>-0.08250219334688401</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>47.63970803071238</v>
+        <v>47.63970813217156</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>24.46382276920145</v>
+        <v>24.46382294520946</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.4005305714480796</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.09945518862831493</v>
+        <v>-0.0994551887264325</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>461.2596177740485</v>
+        <v>461.2596177740491</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>20</v>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>50.53173034343114</v>
+        <v>50.5317303747298</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>10.62384955175526</v>
+        <v>10.6238495746438</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>2.851818566293085</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.07044048147848354</v>
+        <v>0.07044048138036485</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2622,7 +2622,7 @@
         <v>45.90484707074836</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>16.09166021232069</v>
+        <v>16.09166011837508</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.9830428177862458</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.02387868795486116</v>
+        <v>0.02387868809501446</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>47.91113739662757</v>
+        <v>47.91113745847422</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>20.77062009857078</v>
+        <v>20.77062002002396</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1.046944844780225</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>45.52996767493394</v>
+        <v>45.5299675748732</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>28.72846159659593</v>
+        <v>28.72846175073957</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.5969970290769615</v>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>446.1275552542835</v>
+        <v>446.1275552542834</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>11.05</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>53.48868767907326</v>
+        <v>53.48868775839224</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>17.83851637131479</v>
+        <v>17.83851632770369</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.94351239308079</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.01672001995098953</v>
+        <v>0.01672001993697055</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>446.0184672060134</v>
+        <v>446.0184672060135</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>69.7</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>48.90119524669444</v>
+        <v>48.90119531407304</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>15.21305716388626</v>
+        <v>15.21305722505362</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.9174516046541222</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.07487907074761091</v>
+        <v>-0.07487907094385104</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>40.56629876217429</v>
+        <v>40.56629877456848</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>31.6846080064185</v>
+        <v>31.68460792062989</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.7366654226485709</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.1081335552697738</v>
+        <v>-0.1081335553118239</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>58.47485537756555</v>
+        <v>58.47485541475015</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>64.22641151136584</v>
+        <v>64.2264115584602</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.1763728741855054</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.1436329391723479</v>
+        <v>-0.1436329391963704</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>434.7350949140956</v>
+        <v>434.7350949140958</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>107</v>
@@ -2993,7 +2993,7 @@
         <v>51.61039199843174</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>13.14233716754401</v>
+        <v>13.14233712235288</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.5422154285748083</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.2348333998358355</v>
+        <v>0.2348334001161878</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>426.2256036612503</v>
+        <v>426.2256036612502</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>26.5</v>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>48.37519996138513</v>
+        <v>48.37520002038438</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>13.52240632268671</v>
+        <v>13.52240634674843</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>1.036533289575128</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.08582274819667798</v>
+        <v>0.08582274814061394</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,7 +3149,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>46.66568635272273</v>
+        <v>46.66568631565318</v>
       </c>
       <c r="I51" s="2" t="n">
         <v>29.72973555512544</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.1746697747641023</v>
+        <v>-0.1746697746940243</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>43.73047503588652</v>
+        <v>43.73047507842054</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>34.410110244324</v>
+        <v>34.41011030747746</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.5287290176459353</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.09724607070993924</v>
+        <v>-0.09724607078002473</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>408.0867869331105</v>
+        <v>408.0867869331107</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>88.59999999999999</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>52.6241226032864</v>
+        <v>52.62412263076303</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>6.444766288243534</v>
+        <v>6.444766286668123</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.4875341668806329</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.2529556235914483</v>
+        <v>-0.2529556236475159</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>47.4345929121767</v>
+        <v>47.43459298148233</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>36.48648929627024</v>
+        <v>36.48648926027415</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.4503480288655173</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.05008545235478354</v>
+        <v>-0.05008545242487034</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>53.39231258147935</v>
+        <v>53.39231282372943</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>17.52592628712955</v>
+        <v>17.52592633461374</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>1.110544920475465</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.01060223122242689</v>
+        <v>0.01060223118037502</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>399.3025367340298</v>
+        <v>399.3025367340297</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>10.3</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>43.39820066028695</v>
+        <v>43.39820078456646</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>23.09991959203426</v>
+        <v>23.09991960805586</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1.690104392507155</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.02316421768842664</v>
+        <v>0.02316421767441171</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>39.32029422982587</v>
+        <v>39.32029419720229</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>44.38443212941924</v>
+        <v>44.38443221165659</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.26527737954334</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.03832927484595461</v>
+        <v>0.03832927488800508</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
         <v>51.47628324819883</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>9.195140867425428</v>
+        <v>9.195140872499589</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.213837046724031</v>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>388.7671418522368</v>
+        <v>388.7671418522366</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>18.85</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>34.97952221959444</v>
+        <v>34.97952300977602</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>44.88680352530255</v>
+        <v>44.88680351426455</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1.444803384559349</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.0007838579898996334</v>
+        <v>-0.0007838580179355403</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>40.93268069948992</v>
+        <v>40.93268067651901</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>11.74183240172536</v>
+        <v>11.74183244630981</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.7215689761067196</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.417675413804938</v>
+        <v>-0.4176754139451156</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>51.10893496109806</v>
+        <v>51.10893511875808</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>19.23056751969887</v>
+        <v>19.23056761182529</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>1.107740551194117</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.008362932024265073</v>
+        <v>0.008362931884096678</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>49.60348738275516</v>
+        <v>49.60348749241383</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>11.84462254659206</v>
+        <v>11.84462265383216</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>1.268534588509361</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.0382451729630765</v>
+        <v>-0.03824517306119814</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>43.05829138163871</v>
+        <v>43.0582915517282</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>12.82674628956885</v>
+        <v>12.82674623738915</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.4001182870078424</v>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>42.3701167487967</v>
+        <v>42.37011679600633</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>8.319427966574546</v>
+        <v>8.319427580584225</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.4600557741757824</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.2191739813214595</v>
+        <v>0.2191739849658891</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>50.73405691926826</v>
+        <v>50.7340569466283</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>7.973975423213428</v>
+        <v>7.973975485354818</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.5975139833209947</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.0004004808814840428</v>
+        <v>0.0004004809235365874</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>44.89434105419756</v>
+        <v>44.89434106185504</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>34.7786001449895</v>
+        <v>34.77860012876623</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.5454585161494226</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.07383634735732553</v>
+        <v>-0.07383634737134342</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>346.6733874472962</v>
+        <v>346.6733874472952</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>26.65</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>49.5976532914535</v>
+        <v>49.59765344561504</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>28.43959363612493</v>
+        <v>28.43959363310234</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.5393660494386591</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.05352941662611273</v>
+        <v>0.05352941651397894</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,7 +4050,7 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>44.43472540499618</v>
+        <v>44.43472579744652</v>
       </c>
       <c r="I68" s="2" t="n">
         <v>16.63724609672827</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.004043074446452521</v>
+        <v>-0.004043074460464507</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>54.76490287283215</v>
+        <v>54.76490311546614</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>8.820709964488103</v>
+        <v>8.820710048050584</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.3444450285100885</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.00996388305984125</v>
+        <v>0.009963882989755608</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>30.2754452998782</v>
+        <v>30.27544535439078</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>28.26196207568031</v>
+        <v>28.26196199651295</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.7234782411867646</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>43.36351028964666</v>
+        <v>43.36351032575151</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>16.19488793326233</v>
+        <v>16.19488799147967</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.808491582247074</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.02617305409891257</v>
+        <v>-0.02617305416899768</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>41.10513916883784</v>
+        <v>41.10513923354406</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>27.25126446151379</v>
+        <v>27.25126434418434</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.9228546604900439</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.01251598993595038</v>
+        <v>-0.01251599000603373</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>41.64187539323201</v>
+        <v>41.64187540430454</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>15.90290027438911</v>
+        <v>15.90290034858677</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.4808313018780662</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.01251024861324925</v>
+        <v>-0.01251024861885455</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>306.8260899314311</v>
+        <v>306.8260899314309</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>25.2</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>37.30382884942652</v>
+        <v>37.30382886404852</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>14.48436563941315</v>
+        <v>14.48436562863219</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1.663891804908274</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.06593604117833188</v>
+        <v>-0.06593604129046854</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>47.80496237772534</v>
+        <v>47.80496242876569</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>32.49655268292496</v>
+        <v>32.49655268876375</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.407632821778858</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.04664076745402679</v>
+        <v>-0.04664076751009566</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>33.01850203109586</v>
+        <v>33.01850237081086</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>30.00260844242966</v>
+        <v>30.0026085013421</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1.097233452453498</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.06424678573124165</v>
+        <v>-0.06424678578731008</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4530,7 +4530,7 @@
         <v>45.35651942139969</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>33.07498638671085</v>
+        <v>33.07498639151169</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.3913103384926285</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.04513001619581303</v>
+        <v>-0.04513001617899268</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>38.48702325705609</v>
+        <v>38.48702340001114</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>7.617536382793276</v>
+        <v>7.617536367085991</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.6271837785975587</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.00952717578742529</v>
+        <v>0.009527175661270704</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>301.4427551264689</v>
+        <v>301.4427551264691</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>9.859999999999999</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>34.86981319594247</v>
+        <v>34.86981328875386</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>25.36638529354557</v>
+        <v>25.36638541816729</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>1.395196716124667</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.000142484817384686</v>
+        <v>0.0001424848033682036</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4689,7 +4689,7 @@
         <v>34.23088979970008</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>18.41097811400233</v>
+        <v>18.41097809777801</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.7588313416947114</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.00637418885173828</v>
+        <v>0.006374188781653023</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>47.12656670682107</v>
+        <v>47.12656680809518</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>14.17372298714401</v>
+        <v>14.1737229256177</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.9979275133066693</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.003183945382247713</v>
+        <v>0.003183945354215983</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>38.48273887761444</v>
+        <v>38.48273898635008</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>7.9463645255898</v>
+        <v>7.946365366234938</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>1.141736795086661</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.02105877570632486</v>
+        <v>0.02105877556615599</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>50.37570355650195</v>
+        <v>50.37570356125211</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>8.071739603631645</v>
+        <v>8.071739424255387</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>1.591717518967429</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.2737575935030396</v>
+        <v>0.2737575934750045</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>34.63655212079985</v>
+        <v>34.63655192352961</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>13.61785360486242</v>
+        <v>13.61785357122794</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.992951684169262</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.07171242537668543</v>
+        <v>-0.0717124252084802</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>35.74218414138525</v>
+        <v>35.74218412852258</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>11.12301228248422</v>
+        <v>11.12301239054997</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>1.760919502465495</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.01614659393724376</v>
+        <v>-0.01614659394285048</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>280.8215544552973</v>
+        <v>280.8215544552968</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>14.9</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>36.44424994528642</v>
+        <v>36.44425013197098</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>17.67498879254004</v>
+        <v>17.67498879978401</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.5843450739975848</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.007545946962794772</v>
+        <v>-0.007545946948776305</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>279.9882437346843</v>
+        <v>279.9882437346844</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>6.25</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>48.55393282858574</v>
+        <v>48.55393298827664</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>19.11615594113584</v>
+        <v>19.11615594593959</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.2529138567877762</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.01236264550437366</v>
+        <v>0.01236264550156981</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,7 +5110,7 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>36.26359385099953</v>
+        <v>36.26359398506199</v>
       </c>
       <c r="I88" s="2" t="n">
         <v>36.43134016052537</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.007032436169860101</v>
+        <v>-0.00703243618387861</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>275.8085682520794</v>
+        <v>275.8085682520796</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>9.859999999999999</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>40.88061330824178</v>
+        <v>40.88061350871292</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>19.32283039697867</v>
+        <v>19.32283021562689</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.9656777798966892</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.002733308623751617</v>
+        <v>-0.002733308848023405</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>43.43435007362613</v>
+        <v>43.43434962107427</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>16.82255521365153</v>
+        <v>16.82255531475795</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>1.169022783709383</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.04150184485276265</v>
+        <v>0.04150184504494409</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>30.2594886590818</v>
+        <v>30.25948882374236</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>34.58904658087221</v>
+        <v>34.58904659993487</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.6038300506478742</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.009929514370426273</v>
+        <v>0.009929514356408903</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5325,7 +5325,7 @@
         <v>48.73350263634344</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>12.06062426556887</v>
+        <v>12.06062414859582</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.2324904627064758</v>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>269.691343074882</v>
+        <v>269.6913430748816</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>15.3</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>35.73061809196055</v>
+        <v>35.73061852203961</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>30.35315976877381</v>
+        <v>30.35315981427476</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>1.253583202524372</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.02073921310322206</v>
+        <v>-0.02073921313125539</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5431,7 +5431,7 @@
         <v>40.2297815087816</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>40.17210484007352</v>
+        <v>40.17210484439891</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.398569821767086</v>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>255.6636975973329</v>
+        <v>255.6636975973335</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>63.5</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>37.04555218429955</v>
+        <v>37.04555231293152</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>15.17341359534782</v>
+        <v>15.17341357750499</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.3550157074723045</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.2656956509584859</v>
+        <v>-0.2656956511827586</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>50.99084933536099</v>
+        <v>50.99084933066322</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>13.79774724240975</v>
+        <v>13.79774726415332</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>1.009326928468627</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.3789605355213391</v>
+        <v>0.3789605355073216</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>247.0535719787305</v>
+        <v>247.0535719787312</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>69.90000000000001</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>44.13305890940874</v>
+        <v>44.13305899680746</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>13.70675867097003</v>
+        <v>13.7067587393857</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>1.947212138697003</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.01770878467349235</v>
+        <v>0.01770878447725932</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>246.9234449213294</v>
+        <v>246.9234449213295</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>43.8</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>31.78735427169219</v>
+        <v>31.78735372483574</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>24.10910258687021</v>
+        <v>24.10910258792682</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.8609879271902744</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.08278394642341602</v>
+        <v>-0.08278394561043367</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>46.32820850865157</v>
+        <v>46.3282083954993</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>13.43046753543922</v>
+        <v>13.43046749088098</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4522391118085424</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.004306510590113166</v>
+        <v>-0.004306510576095615</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>38.27339308707172</v>
+        <v>38.27339333551261</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>18.31161572625699</v>
+        <v>18.31161574741834</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.6835417548362436</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.0151198826557355</v>
+        <v>-0.01511988269778535</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>234.3729286086362</v>
+        <v>234.3729286086365</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>32.05</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>37.17682643631351</v>
+        <v>37.1768269632432</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>10.08564701099007</v>
+        <v>10.08564705762232</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.7015852638147142</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.03795846226011274</v>
+        <v>-0.03795846227413339</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>232.7062305274769</v>
+        <v>232.7062305274796</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>96.7</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>31.06818707941413</v>
+        <v>31.0681873661396</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>18.68040907923018</v>
+        <v>18.68040913097878</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>1.711676728001756</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.3157175437548441</v>
+        <v>-0.3157175438669865</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>231.6225511311849</v>
+        <v>231.6225511311848</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>615</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>33.30214368564765</v>
+        <v>33.3021437784537</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>12.71618488121825</v>
+        <v>12.71618488895323</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5237464880521181</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-7.221732687026851</v>
+        <v>-7.221732692913974</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>41.53060187775376</v>
+        <v>41.53060200354995</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>24.7414289684885</v>
+        <v>24.74142898198684</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.4976793908482958</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.05860629757175465</v>
+        <v>-0.05860629758577153</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6014,7 +6014,7 @@
         <v>51.30613010717237</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>8.699330880273015</v>
+        <v>8.699330913651206</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.534455435045157</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>38.00230946826648</v>
+        <v>38.00230951115786</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>17.1794584639681</v>
+        <v>17.17945850692499</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>2.103509245009634</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.003937246065421091</v>
+        <v>0.003937246079439446</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>42.23756932353022</v>
+        <v>42.23756941128819</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>9.796564315084856</v>
+        <v>9.796564411579839</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.8919521866451359</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.6151077143283727</v>
+        <v>-0.6151077157300788</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>216.5131984072286</v>
+        <v>216.5131984072287</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>13.3</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>39.13823110943726</v>
+        <v>39.13823128478966</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>12.03879517598908</v>
+        <v>12.03879509252391</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>1.036579126426111</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.001762770009335432</v>
+        <v>0.001762769995320615</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>205.4639235773386</v>
+        <v>205.4639235773384</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>21.55</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>47.08398949244717</v>
+        <v>47.08398967086807</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>7.494613851280223</v>
+        <v>7.494613856271698</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.7250902417192936</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.009910535161537462</v>
+        <v>0.009910534923249281</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>201.2126428627769</v>
+        <v>201.212642862777</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>26</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>35.17635284514378</v>
+        <v>35.17635332073309</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>31.24519962925976</v>
+        <v>31.24519970597999</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.3988081913507854</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.00938773146843086</v>
+        <v>0.0093877312721935</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>194.9523194066122</v>
+        <v>194.9523194066118</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>39.95</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>43.65617313912831</v>
+        <v>43.65617323297415</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.56211252246812</v>
+        <v>17.56211257893873</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.5312389084996308</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.01970664813471337</v>
+        <v>0.01970664803659333</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>193.7034867605876</v>
+        <v>193.7034867605865</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>28.9</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>38.251120029319</v>
+        <v>38.25111964136786</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>22.97816382511045</v>
+        <v>22.97816452947856</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.5314132171035814</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.3378993239871319</v>
+        <v>-0.3378993235385866</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>192.9307045529357</v>
+        <v>192.9307045529352</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>9.710000000000001</v>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>29.31252516957822</v>
+        <v>29.31252522539661</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>22.01298880478296</v>
+        <v>22.01298882918486</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>1.360898114894205</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.01691312567572451</v>
+        <v>-0.01691312568973949</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>38.3210174005151</v>
+        <v>38.32101738765611</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>21.88645097900668</v>
+        <v>21.88645103429687</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.001584990708859</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>40.21898436341603</v>
+        <v>40.21898445804143</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>19.15769523305918</v>
+        <v>19.15769534453129</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.1910303369452782</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.01499404685069336</v>
+        <v>0.01499404683667602</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.8957435396395</v>
+        <v>39.8957437250638</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>22.60886457362271</v>
+        <v>22.60886461090679</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.5399184266849736</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.0942743995079792</v>
+        <v>-0.09427439960609577</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>182.901016227601</v>
+        <v>182.9010162276014</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>6.22</v>
@@ -6650,7 +6650,7 @@
         <v>37.36424647422256</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>23.51100455219949</v>
+        <v>23.51100469886644</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>1.122346288879889</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.01097314850539313</v>
+        <v>-0.0109731485025901</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>181.8618183480426</v>
+        <v>181.8618183480429</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>74.3</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>20.77512345552299</v>
+        <v>20.77512239411307</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>36.12172657205576</v>
+        <v>36.1217271163828</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.7811844471055056</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.3064339964838934</v>
+        <v>-0.3064339953625219</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>172.622065604318</v>
+        <v>172.6220656043153</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>12</v>
@@ -6753,7 +6753,7 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>40.41731719505214</v>
+        <v>40.41731717145799</v>
       </c>
       <c r="I119" s="2" t="n">
         <v>20.99784949065089</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.05279314737344756</v>
+        <v>-0.05279314735943069</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,7 +6806,7 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>38.74514951413121</v>
+        <v>38.74514951219163</v>
       </c>
       <c r="I120" s="2" t="n">
         <v>17.09814368084951</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>50.06999611718037</v>
+        <v>50.06999625104883</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>5.946345208951548</v>
+        <v>5.946344482879645</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.5098654521723434</v>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>158.39324731357</v>
+        <v>158.3932473135714</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>9.01</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>32.40390734905704</v>
+        <v>32.40390756516165</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>15.84219300251613</v>
+        <v>15.84219298304317</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>1.381537630934448</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.02329689750084775</v>
+        <v>-0.02329689754289752</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>157.5768665362972</v>
+        <v>157.5768665362973</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>14.4</v>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>43.58614458480404</v>
+        <v>43.58614464424703</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>15.99865273214649</v>
+        <v>15.99865275079692</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.7138346245074088</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.04832510574995136</v>
+        <v>0.04832510573593579</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>42.95216474024279</v>
+        <v>42.95216461466087</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>15.94059467302017</v>
+        <v>15.94059473872347</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.3061135049663243</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.02715903398230293</v>
+        <v>0.0271590339402525</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>139.4856444413938</v>
+        <v>139.4856444413934</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>18.65</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>38.71151293968626</v>
+        <v>38.71151304456053</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>10.4538930990547</v>
+        <v>10.45389313396732</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.6394762684124387</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.002725307383973807</v>
+        <v>-0.002725307454058079</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>139.4479191146526</v>
+        <v>139.4479191146521</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>8.09</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>42.24321417403042</v>
+        <v>42.24321424124142</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>13.37833829015054</v>
+        <v>13.37833818066517</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.4283024881512028</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>0.003163794723434196</v>
+        <v>0.003163794720629075</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>8.101614084452024</v>
+        <v>8.101614134512275</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>32.26218604406749</v>
+        <v>32.26218610488139</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.08126407941833376</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>44.76535378377109</v>
+        <v>44.76535383078174</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>6.053047195481095</v>
+        <v>6.053047258460385</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.8043434055369213</v>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>35.60669350462861</v>
+        <v>35.60669360864836</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>21.45247887624866</v>
+        <v>21.45247884121664</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>0.3759249138092666</v>
@@ -7301,7 +7301,7 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>-0.0352602752841959</v>
+        <v>-0.03526027545239968</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7322,7 +7322,7 @@
         <v/>
       </c>
       <c r="D130" s="2" t="n">
-        <v>105.1629217276462</v>
+        <v>105.1629217276461</v>
       </c>
       <c r="E130" s="2" t="n">
         <v>35.2</v>
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>36.68310713789047</v>
+        <v>36.68310752702267</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>13.32351274331679</v>
+        <v>13.32351266204702</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.8476287377514268</v>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>42.86656468197072</v>
+        <v>42.86656471572707</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>17.2902323758677</v>
+        <v>17.29023238319868</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.4184158987861103</v>
@@ -7428,7 +7428,7 @@
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>84.39037585176541</v>
+        <v>84.39037585176543</v>
       </c>
       <c r="E132" s="2" t="n">
         <v>27.6</v>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>37.83218397245656</v>
+        <v>37.83218399930594</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>17.80643321058857</v>
+        <v>17.80643325140756</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.7334442338185182</v>
@@ -7481,7 +7481,7 @@
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>83.83811406728192</v>
+        <v>83.83811406728209</v>
       </c>
       <c r="E133" s="2" t="n">
         <v>0</v>
@@ -7495,7 +7495,7 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>37.10901102455061</v>
+        <v>37.10901102631047</v>
       </c>
       <c r="I133" s="2" t="n">
         <v>8.465557602412245</v>
@@ -7513,7 +7513,7 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>-2.825112366861719</v>
+        <v>-2.825112367001884</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>

</xml_diff>